<commit_message>
release: module three buyer roster, backup environments and parallel creation in v0.7.0
- 固定采购员名单（新刚-XG/志恒-ZH/康德-KD/宇航-YH）与英文代号环境命名
- 新增备用/测试环境模式（不绑号，写固定备注，结果清单导出）
- 绑号与备用建环境并行执行（默认 5 并发，设置可调 1-10）
- 内置默认代理提取链接与分组默认选中，同事端零配置
- Cookie 登录域站点校验（预览+正式执行双重整批拒收）
- 同名环境收养防护与进度即时刷新
</commit_message>
<xml_diff>
--- a/examples/buyer-import-template.xlsx
+++ b/examples/buyer-import-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Ra80129bca7a8480d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R6d1ed1818e834630"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rbffc3e4d31a74c56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="Racf0a6a9367249f3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,7 +14,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="5">
+  <x:fonts count="7">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -41,8 +41,19 @@
       <x:color rgb="FF1F2937"/>
       <x:name val="Aptos"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Aptos"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -64,8 +75,18 @@
         <x:fgColor rgb="FFCCFBF1"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8FAFC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF147D74"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="15">
+  <x:borders count="16">
     <x:border/>
     <x:border>
       <x:right style="thin">
@@ -198,13 +219,27 @@
       </x:top>
       <x:bottom style="thin">
         <x:color rgb="FFCBD5E1"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FF0F5F59"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FF0F5F59"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF0F5F59"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF0F5F59"/>
       </x:bottom>
     </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="39">
+  <x:cellXfs count="60">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -277,6 +312,63 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -487,72 +579,86 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="12" t="str">
+      <x:c r="A1" s="59" t="str">
+        <x:v>邮箱账号</x:v>
+      </x:c>
+      <x:c r="B1" s="59" t="str">
+        <x:v>密码</x:v>
+      </x:c>
+      <x:c r="C1" s="59" t="str">
+        <x:v>接码Key链接</x:v>
+      </x:c>
+      <x:c r="D1" s="59" t="str">
+        <x:v>Cookie</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="28" customHeight="1">
+      <x:c r="A2" s="48" t="str">
         <x:v>buyer01@example.test</x:v>
       </x:c>
-      <x:c r="B1" s="13" t="str">
+      <x:c r="B2" s="48" t="str">
         <x:v>Example-Password-Only</x:v>
       </x:c>
-      <x:c r="C1" s="13" t="str">
+      <x:c r="C2" s="48" t="str">
         <x:v>https://codes.example.test/key?orderNo=0000000000000001</x:v>
       </x:c>
-      <x:c r="D1" s="14" t="str">
+      <x:c r="D2" s="48" t="str">
         <x:v>[{"name":"language","value":"es","domain":".example.test"},{"name":"session","value":"FAKE-SESSION-01","domain":".example.test"}]</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="28" customHeight="1">
-      <x:c r="A2" s="15" t="str">
+    <x:row r="3" ht="28" customHeight="1">
+      <x:c r="A3" s="48" t="str">
         <x:v>buyer02@example.test</x:v>
       </x:c>
-      <x:c r="B2" s="16" t="str">
+      <x:c r="B3" s="48" t="str">
         <x:v>Example-Password-Only</x:v>
       </x:c>
-      <x:c r="C2" s="16" t="str">
+      <x:c r="C3" s="48" t="str">
         <x:v>https://codes.example.test/key?orderNo=0000000000000002</x:v>
       </x:c>
-      <x:c r="D2" s="17" t="str">
+      <x:c r="D3" s="48" t="str">
         <x:v>[{"name":"language","value":"es","domain":".example.test"},{"name":"session","value":"FAKE-SESSION-02","domain":".example.test"}]</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="28" customHeight="1">
-      <x:c r="A3" s="15" t="str">
+    <x:row r="4" ht="28" customHeight="1">
+      <x:c r="A4" s="48" t="str">
         <x:v>buyer03@example.test</x:v>
       </x:c>
-      <x:c r="B3" s="16" t="str">
+      <x:c r="B4" s="48" t="str">
         <x:v>Example-Password-Only</x:v>
       </x:c>
-      <x:c r="C3" s="16" t="str">
+      <x:c r="C4" s="48" t="str">
         <x:v>https://codes.example.test/key?orderNo=0000000000000003</x:v>
       </x:c>
-      <x:c r="D3" s="17" t="str">
+      <x:c r="D4" s="48" t="str">
         <x:v>[{"name":"language","value":"es","domain":".example.test"},{"name":"session","value":"FAKE-SESSION-03","domain":".example.test"}]</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="15" t="str">
+    <x:row r="5" ht="28" customHeight="1">
+      <x:c r="A5" s="48" t="str">
         <x:v>buyer04@example.test</x:v>
       </x:c>
-      <x:c r="B4" s="16" t="str">
+      <x:c r="B5" s="48" t="str">
         <x:v>Example-Password-Only</x:v>
       </x:c>
-      <x:c r="C4" s="16" t="str">
+      <x:c r="C5" s="48" t="str">
         <x:v>https://codes.example.test/key?orderNo=0000000000000004</x:v>
       </x:c>
-      <x:c r="D4" s="17" t="str">
+      <x:c r="D5" s="48" t="str">
         <x:v>[{"name":"language","value":"es","domain":".example.test"},{"name":"session","value":"FAKE-SESSION-04","domain":".example.test"}]</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="28" customHeight="1">
-      <x:c r="A5" s="18" t="str">
+    <x:row r="6">
+      <x:c r="A6" s="50" t="str">
         <x:v>buyer05@example.test</x:v>
       </x:c>
-      <x:c r="B5" s="19" t="str">
+      <x:c r="B6" s="50" t="str">
         <x:v>Example-Password-Only</x:v>
       </x:c>
-      <x:c r="C5" s="19" t="str">
+      <x:c r="C6" s="50" t="str">
         <x:v>https://codes.example.test/key?orderNo=0000000000000005</x:v>
       </x:c>
-      <x:c r="D5" s="20" t="str">
+      <x:c r="D6" s="50" t="str">
         <x:v>[{"name":"language","value":"es","domain":".example.test"},{"name":"session","value":"FAKE-SESSION-05","domain":".example.test"}]</x:v>
       </x:c>
     </x:row>
@@ -585,44 +691,44 @@
         <x:v>Requirement</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="30" customHeight="1">
+    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A4" s="36" t="str">
         <x:v>Worksheet</x:v>
       </x:c>
       <x:c r="B4" s="36" t="str">
-        <x:v>Put import rows in Sheet1. Start at row 1 and do not add headers.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="30" customHeight="1">
+        <x:v>Keep the header row in the Xynigo template; data starts on row 2. Imports also accept recognized vendor files without a header.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="37" t="str">
         <x:v>Column A</x:v>
       </x:c>
       <x:c r="B5" s="37" t="str">
-        <x:v>Buyer email address</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="30" customHeight="1">
+        <x:v>Buyer email address (template header: 邮箱账号)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="37" t="str">
         <x:v>Column B</x:v>
       </x:c>
       <x:c r="B6" s="37" t="str">
-        <x:v>Account password</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="30" customHeight="1">
+        <x:v>Account password (template header: 密码)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="37" t="str">
         <x:v>Column C</x:v>
       </x:c>
       <x:c r="B7" s="37" t="str">
-        <x:v>Verification-code URL supplied by your authorized provider</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="30" customHeight="1">
+        <x:v>Verification-code URL supplied by your authorized provider (template header: 接码Key链接)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="37" t="str">
         <x:v>Column D</x:v>
       </x:c>
       <x:c r="B8" s="37" t="str">
-        <x:v>Cookie JSON string copied without reformatting</x:v>
+        <x:v>Cookie JSON string copied without reformatting (template header: Cookie)</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">

</xml_diff>